<commit_message>
Body and animations overhaul
</commit_message>
<xml_diff>
--- a/Docs/B-15 Art asset list.xlsx
+++ b/Docs/B-15 Art asset list.xlsx
@@ -321,7 +321,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="42.25" customWidth="1" style="2" min="2" max="2"/>
@@ -398,7 +398,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>SK_Valhalla_Body</t>
+          <t>SKM_MHC_ValhallaBase (MetaHuman body + face)</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -413,7 +413,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Existing (replaced)</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -423,17 +423,17 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>Opus 5.5 + Blender MCP: organic body (base mesh for all humanoid races)</t>
+          <t>MetaHuman Creator in UE 5.8 (MetaHumanCharacter plugin), Optimized / Medium build</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>CC0 skin/cloth textures or procedural bake</t>
+          <t>MetaHuman skin (baked by the build)</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>Rig on SK_Valhalla_Skeleton; weights hand-tuned</t>
+          <t>metahuman_base_skel; face mesh follows the body by leader pose</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
@@ -448,7 +448,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>Done 2026-09-23 (Fable 5.1): Organic body: parametric shells -&gt; voxel remesh -&gt; scripted sculpt -&gt; QuadriFlow retopo (wave2_body.py), scripted weights on the unchanged skeleton (same 24 joints, sockets). 8,844 tris. Procedural skin set SkinBase (baked, own work); runtime BaseColor tint still works. Race_Stocky/Slender shape keys in .blend/glb only.</t>
+          <t>Done 2026-09-23 (Opus 5.5): Replaced the Fable 5.1 organic body with the MetaHuman base MHC_ValhallaBase, nude in underwear, drawn at 122/180.3 scale, facing +Y. Content in /Game/Valhalla/Characters/MetaHuman/ (~455 MB with Build + Export). The Fable body remains as valhalla.Visual.BodyProfile 0. The Paragon Gideon trial body was archived outside the repo (Valhalla-archive/ParagonGideon_2026-09-23). Armour and hair must be rebuilt on metahuman_base_skel (A-002..A-020).</t>
         </is>
       </c>
     </row>
@@ -505,12 +505,12 @@
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Clumped hair cards on the new cranium, vertex-colour roots (wave2_hair.py). 5,022 tris. HairStrands procedural set.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Clumped hair cards on the new cranium, vertex-colour roots (wave2_hair.py). 5,022 tris. HairStrands procedural set.</t>
         </is>
       </c>
     </row>
@@ -567,12 +567,12 @@
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Short clumped hair with fringe. 4,590 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L4" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Short clumped hair with fringe. 4,590 tris.</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Scalp patch on skin material. 972 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L5" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Scalp patch on skin material. 972 tris.</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="K6" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather jerkin with straps, studs, belt. 1,252 tris. ambientCG Leather028.</t>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather jerkin with straps, studs, belt. 1,252 tris. ambientCG Leather028.</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Chain shirt (ambientCG Chainmail004) with cloth tabard. 1,712 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L7" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Chain shirt (ambientCG Chainmail004) with cloth tabard. 1,712 tris.</t>
         </is>
       </c>
     </row>
@@ -815,12 +815,12 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Blue robe, bell sleeves, rope belt (ambientCG Fabric032 tinted). 2,488 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L8" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Blue robe, bell sleeves, rope belt (ambientCG Fabric032 tinted). 2,488 tris.</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth trousers with leather patches. 1,784 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L9" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth trousers with leather patches. 1,784 tris.</t>
         </is>
       </c>
     </row>
@@ -939,12 +939,12 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Plate cuisses/greaves with knee cops (ambientCG Metal009). 1,704 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L10" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Plate cuisses/greaves with knee cops (ambientCG Metal009). 1,704 tris.</t>
         </is>
       </c>
     </row>
@@ -1001,12 +1001,12 @@
       </c>
       <c r="K11" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Robe skirt (stretches between legs rather than swinging). 1,008 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L11" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Robe skirt (stretches between legs rather than swinging). 1,008 tris.</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1063,12 @@
       </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather boots. 1,576 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L12" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather boots. 1,576 tris.</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1125,12 @@
       </c>
       <c r="K13" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Plate sabatons. 1,528 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L13" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Plate sabatons. 1,528 tris.</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth slippers. 856 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L14" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth slippers. 856 tris.</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="K15" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather bracers. 1,568 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L15" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather bracers. 1,568 tris.</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Gauntlets with knuckle lames. 1,424 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L16" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Gauntlets with knuckle lames. 1,424 tris.</t>
         </is>
       </c>
     </row>
@@ -1373,12 +1373,12 @@
       </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth wraps (stacked bands). 1,696 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L17" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Cloth wraps (stacked bands). 1,696 tris.</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1435,12 @@
       </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Full helm, T-visor, crest. 960 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L18" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Full helm, T-visor, crest. 960 tris.</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather hood with mantle (stiff). 1,140 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L19" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Leather hood with mantle (stiff). 1,140 tris.</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Wizard hat with bent cone. 868 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L20" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Wizard hat with bent cone. 868 tris.</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="K21" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Wool cloak (stiff sheet, no cloth sim). 664 tris.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L21" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the version below is skinned to SK_Valhalla_Skeleton, cannot follow metahuman_base_skel and is hidden on the MetaHuman body. | Previous: Done 2026-09-23 (Fable 5.1): Built by wave2_armour.py: ray-cast fitted to the new body, skinned with the body weights, Race_Stocky/Slender keys (not imported: morph targets off). Wool cloak (stiff sheet, no cloth sim). 664 tris.</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Animations (7): Idle Walk Attack Shoot Cast Hit Death</t>
+          <t>Animations: Idle Walk Jog Attack Hit Death (MetaHuman)</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Existing (replaced)</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="I30" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: scripted keyframe animation on SK_Valhalla_Skeleton</t>
+          <t>Retargeted from the UE5 Mannequin (IK_Manny -&gt; IK_MH_ValhallaBase) + hand-keyed fixes (Tools/anim_authoring)</t>
         </is>
       </c>
       <c r="J30" s="1" t="inlineStr">
@@ -2184,11 +2184,11 @@
       </c>
       <c r="L30" s="1" t="inlineStr">
         <is>
-          <t>Done 2026-09-23 (Fable 5.1): Re-keyed by wave2_anims.py (FK + planted-foot leg solver), same names, 30 fps: Idle 2.0 s loop, Walk 0.667 s loop (matches 122 cm/s), Attack/Shoot 0.667 s, Cast 0.8 s, Hit 0.4 s, Death 1.2 s hold. No gameplay timing depends on length.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
+          <t>Done 2026-09-23 (Opus 5.5): MetaHuman set in /Game/Valhalla/Characters/MetaHuman/Animations. Idle MH_MM_Idle re-posed relaxed (arms at the sides, hands at rest). Walk MH_MF_Unarmed_Walk_Fwd and Jog MH_MF_Unarmed_Jog_Fwd, play rate matched to speed. Unarmed attack MH_MM_Attack_01. Hit MH_MM_HitReact_Front_Lgt_01 on an additive layer (fixed the combat flicker). Death MH_MM_Death_Front_01. Shoot and Cast moved to A-088/A-091. Mannequin source archived (Valhalla-archive/UE5Mannequins_2026-09-23). Fable 5.1 clips kept for BodyProfile 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" s="2">
       <c r="A31" s="1" t="inlineStr">
         <is>
           <t>A-030</t>
@@ -2241,12 +2241,12 @@
       </c>
       <c r="K31" s="1" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Done 2026-09-23 (Fable 5.1): Authored and imported (A_Run, A_Sit, A_Emote_Wave/Cheer/Bow, A_Attack2H, A_Block, A_Dodge); added to character_import.ANIMATIONS. NOT wired into gameplay yet - needs EValhallaAnim entries, run locomotion blend, /sit &amp; emote commands, TwoHand attack cycle, Block/Dodge on combat events.</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L31" s="0" t="inlineStr">
+        <is>
+          <t>Rework for the MetaHuman body in progress (2026-09-23 (Opus 5.5)): the clips below are on SK_Valhalla_Skeleton; MetaHuman versions are hand-keyed in Tools/anim_authoring. Still not wired into gameplay. | Previous: Done 2026-09-23 (Fable 5.1): Authored and imported (A_Run, A_Sit, A_Emote_Wave/Cheer/Bow, A_Attack2H, A_Block, A_Dodge); added to character_import.ANIMATIONS. NOT wired into gameplay yet - needs EValhallaAnim entries, run locomotion blend, /sit &amp; emote commands, TwoHand attack cycle, Block/Dodge on combat events.</t>
         </is>
       </c>
     </row>
@@ -5676,6 +5676,316 @@
       <c r="L88" s="1" t="inlineStr">
         <is>
           <t>Done 2026-09-22: Opaque glossy water, two panning normals, fresnel deep/edge colour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" s="2">
+      <c r="A89" s="1" t="inlineStr">
+        <is>
+          <t>A-088</t>
+        </is>
+      </c>
+      <c r="B89" s="1" t="inlineStr">
+        <is>
+          <t>Weapon attacks (MetaHuman): MH_Attack_Sword / _Dagger / _Mace / _Staff / _Bow</t>
+        </is>
+      </c>
+      <c r="C89" s="1" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="D89" s="1" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+      <c r="E89" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F89" s="1" t="inlineStr">
+        <is>
+          <t>Auto-attack with a weapon (AttackAnimForWeapon, by weaponStyle)</t>
+        </is>
+      </c>
+      <c r="G89" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H89" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I89" s="1" t="inlineStr">
+        <is>
+          <t>Hand-keyed in Python (Tools/anim_authoring/author.py)</t>
+        </is>
+      </c>
+      <c r="J89" s="1" t="inlineStr">
+        <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="K89" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L89" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (Opus 5.5): One swing per weapon style: sword slash, dagger thrust, mace overhead, staff two-hand strike, bow draw-and-loose (Shoot). Unarmed stays MH_MM_Attack_01. items.json iron_dagger weaponStyle = dagger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" s="2">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>A-089</t>
+        </is>
+      </c>
+      <c r="B90" s="1" t="inlineStr">
+        <is>
+          <t>Stance poses: MHP_GripR / MHP_GripL / MHP_ShieldArm</t>
+        </is>
+      </c>
+      <c r="C90" s="1" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="D90" s="1" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+      <c r="E90" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F90" s="1" t="inlineStr">
+        <is>
+          <t>Any character holding a weapon or shield</t>
+        </is>
+      </c>
+      <c r="G90" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I90" s="1" t="inlineStr">
+        <is>
+          <t>Hand-keyed; layered per branch in ValhallaAnimInstance (HandLayer)</t>
+        </is>
+      </c>
+      <c r="J90" s="1" t="inlineStr">
+        <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="K90" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L90" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (Opus 5.5): Fingers close on the weapon in the right hand (or the left for a bow), and the forearm comes up to carry a shield. Blended over idle, walk and attacks. Grip transforms for sword, staff, bow and shield are in ValhallaVisuals GripFrame (Tools/anim_authoring grips).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" s="2">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>A-090</t>
+        </is>
+      </c>
+      <c r="B91" s="1" t="inlineStr">
+        <is>
+          <t>Bow skill hold: MH_Bow_Draw / MH_Bow_Release</t>
+        </is>
+      </c>
+      <c r="C91" s="1" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="D91" s="1" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+      <c r="E91" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F91" s="1" t="inlineStr">
+        <is>
+          <t>Skills with castAnimation "bow" (ranger_aimed_shot)</t>
+        </is>
+      </c>
+      <c r="G91" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I91" s="1" t="inlineStr">
+        <is>
+          <t>Hand-keyed (author.py)</t>
+        </is>
+      </c>
+      <c r="J91" s="1" t="inlineStr">
+        <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="K91" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L91" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (Opus 5.5): Draws the bow and holds at full draw for the cast time, then looses when the cast completes. Skill field castAnimation (skills.json, editor checkbox "Bow Draw While Casting"). Candidates for later: Snipe, Multi-Shot, Serpent Arrow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" s="2">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>A-091</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr">
+        <is>
+          <t>Casts: MH_Cast_Instant(_Staff), MH_Cast_Channel(_Staff), MH_Cast_Release(_Staff)</t>
+        </is>
+      </c>
+      <c r="C92" s="1" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="D92" s="1" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+      <c r="E92" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F92" s="1" t="inlineStr">
+        <is>
+          <t>Every spell</t>
+        </is>
+      </c>
+      <c r="G92" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I92" s="1" t="inlineStr">
+        <is>
+          <t>Hand-keyed (author.py)</t>
+        </is>
+      </c>
+      <c r="J92" s="1" t="inlineStr">
+        <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="K92" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L92" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (Opus 5.5): Replaced the Gideon cast. Open-hand and staff variants: a looping channel while the cast bar runs, a release when it completes, and an instant cast for spells with no cast time. Works with a mace + buckler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" s="2">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>A-092</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="inlineStr">
+        <is>
+          <t>MetaHuman retarget + authoring tools (IK_MH_ValhallaBase, Tools/anim_authoring)</t>
+        </is>
+      </c>
+      <c r="C93" s="1" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="D93" s="1" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+      <c r="E93" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F93" s="1" t="inlineStr">
+        <is>
+          <t>Animation pipeline</t>
+        </is>
+      </c>
+      <c r="G93" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I93" s="1" t="inlineStr">
+        <is>
+          <t>IK Rig / IK Retargeter from Python; FK keyframe authoring</t>
+        </is>
+      </c>
+      <c r="J93" s="1" t="inlineStr">
+        <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="K93" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L93" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (Opus 5.5): Tools/anim_authoring: skeleton maths, rig, keyframe engine (Catmull-Rom), UE read/write of AnimSequences, retarget script. IK_MH_ValhallaBase is the target rig; run_op_initial_setup is required on every op or the pelvis lands at 0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HUD overhaul and updated art
</commit_message>
<xml_diff>
--- a/Docs/B-15 Art asset list.xlsx
+++ b/Docs/B-15 Art asset list.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>Done 2026-09-23 (Opus 5.5): Replaced the Fable 5.1 organic body with the MetaHuman base MHC_ValhallaBase, nude in underwear, drawn at 122/180.3 scale, facing +Y. Content in /Game/Valhalla/Characters/MetaHuman/ (~455 MB with Build + Export). The Fable body remains as valhalla.Visual.BodyProfile 0. The Paragon Gideon trial body was archived outside the repo (Valhalla-archive/ParagonGideon_2026-09-23). Armour and hair must be rebuilt on metahuman_base_skel (A-002..A-020).</t>
+          <t>Done 2026-09-23 (Opus 5.5): Replaced the Fable 5.1 organic body with the MetaHuman base MHC_ValhallaBase, nude in underwear, drawn at 122/180.3 scale, facing +Y. Content in /Game/Valhalla/Characters/MetaHuman/ (~455 MB with Build + Export). The Fable body remains as valhalla.Visual.BodyProfile 0. The Paragon Gideon trial body was archived outside the repo (Valhalla-archive/ParagonGideon_2026-09-23). Armour and hair were rebuilt on metahuman_base_skel (A-002..A-020).</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="L31" s="0" t="inlineStr">
         <is>
-          <t>Done 2026-09-23 (Opus 5.5): MH_Sit (0.8 s down to the ground, holds the last frame), MH_Emote_Wave, MH_Emote_Cheer, MH_Emote_Bow, MH_Attack_2H (two-handed overhead chop, left hand on the grip below the right), MH_Block (shield raised to the face, weapon across; the forearm is rolled so the shield faces forward), MH_Dodge (in-place sidestep). Run = MH_MF_Unarmed_Jog_Fwd, already the jog in locomotion. Still NOT wired into gameplay: needs EValhallaAnim entries, /sit and emote commands, a TwoHand weapon style, and Block/Dodge on combat events. | Fable 5.1: Done 2026-09-23 (Fable 5.1): Authored and imported (A_Run, A_Sit, A_Emote_Wave/Cheer/Bow, A_Attack2H, A_Block, A_Dodge); added to character_import.ANIMATIONS. NOT wired into gameplay yet - needs EValhallaAnim entries, run locomotion blend, /sit &amp; emote commands, TwoHand attack cycle, Block/Dodge on combat events.</t>
+          <t>Done 2026-09-23 (Opus 5.5): MH_Sit (0.8 s down to the ground, holds the last frame), MH_Emote_Wave, MH_Emote_Cheer, MH_Emote_Bow, MH_Attack_2H (two-handed overhead chop, left hand on the grip below the right), MH_Block (shield raised to the face, weapon across; the forearm is rolled so the shield faces forward), MH_Dodge (in-place sidestep). Run = MH_MF_Unarmed_Jog_Fwd, already the jog in locomotion. Wired 2026-09-23: chat /sit (toggles) /stand /wave /cheer /bow (ServerEmote; sitting replicates, emotes multicast; moving, casting, attacking or dying stands you up); A_Block / A_Dodge play on the defender of a blocked / dodged blow (not over a swing); weaponStyle "greatsword" uses MH_Attack_2H and is two-handed. Sitting regen and Meditate: backlog B-18. | Fable 5.1: Done 2026-09-23 (Fable 5.1): Authored and imported (A_Run, A_Sit, A_Emote_Wave/Cheer/Bow, A_Attack2H, A_Block, A_Dodge); added to character_import.ANIMATIONS. NOT wired into gameplay yet - needs EValhallaAnim entries, run locomotion blend, /sit &amp; emote commands, TwoHand attack cycle, Block/Dodge on combat events.</t>
         </is>
       </c>
     </row>
@@ -2717,12 +2717,12 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>Ground surface</t>
+          <t>Opus 5.5 + Blender MCP: 64 cm tiles, 7.3 cm top as the first pass</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>CC0 tiling material</t>
+          <t>CC0: ambientCG Ground080 (DesertSand) + Ground097 (SandRipples)</t>
         </is>
       </c>
       <c r="I39" s="1" t="inlineStr">
@@ -2737,7 +2737,12 @@
       </c>
       <c r="K39" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L39" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): MI_SandBlend on M_ValhallaGroundBlend: DesertSand, with patches of wind-rippled SandRipples painted by vertex colour on B and C (faded out at every tile edge, so any tile meets any other). World-aligned, 200 / 150 cm. Tint 0.74/0.69/0.62.</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2779,12 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural terrain</t>
+          <t>Opus 5.5 + Blender MCP: procedural mound</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>CC0 sand</t>
+          <t>CC0 sand (MI_SandBlend)</t>
         </is>
       </c>
       <c r="I40" s="1" t="inlineStr">
@@ -2794,7 +2799,12 @@
       </c>
       <c r="K40" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L40" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): In the Desert every dune is its own actor on top of a sand tile (scaled 1.1-1.6, diagonal chains), so the square first-pass tile showed as a raised square. Now only the mound: round, 0.96 m across (neighbours overlap into bumpy ridges along either diagonal), gentle windward side and steep slip face, rim 2 cm up so it rises out of the sand with no edge. Ripples on the upper windward slope.</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2841,12 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>Ground surface</t>
+          <t>Opus 5.5 + Blender MCP: 64 cm tile, 6.2 cm top</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>CC0 tiling material</t>
+          <t>CC0: Poly Haven dry_ground_01 (CrackedEarth)</t>
         </is>
       </c>
       <c r="I41" s="1" t="inlineStr">
@@ -2851,7 +2861,12 @@
       </c>
       <c r="K41" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L41" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): MI_CrackedBlend: cracked clay pan in the middle, drifted sand creeping in at the edges (half and half at the very edge, so a cluster of pans reads as one). Warmer tint than the grey scan.</t>
         </is>
       </c>
     </row>
@@ -2888,12 +2903,12 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: organic model</t>
+          <t>Opus 5.5 + Blender MCP: fluted stems (ribbed lathe along a path)</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>Procedural / CC0</t>
+          <t>Procedural rib texture (wave3_cactus_texture.py): areoles and spines on each rib crest</t>
         </is>
       </c>
       <c r="I42" s="1" t="inlineStr">
@@ -2908,7 +2923,12 @@
       </c>
       <c r="K42" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L42" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): A: saguaro-like column with two elbowed arms, 10 ribs. B: barrel cactus with a pup and three flowers (MI_CactusFlower). One texture repeat per rib across and per metre up. First-pass bounds kept.</t>
         </is>
       </c>
     </row>
@@ -2945,12 +2965,12 @@
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural tree + frond cards</t>
+          <t>Opus 5.5 + Blender MCP: ringed leaning trunk + 13 frond cards</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>CC0 bark + leaf atlas</t>
+          <t>CC0: Poly Haven palm_bark; frond texture procedural (wave3_palm_texture.py)</t>
         </is>
       </c>
       <c r="I43" s="1" t="inlineStr">
@@ -2965,7 +2985,12 @@
       </c>
       <c r="K43" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L43" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): Trunk with leaf-scar rings and flared foot (MI_PalmBark), crown boot, hanging fruit (MI_Coconut), 9 drooping + 4 rising fronds folded along the rachis; MI_PalmFrond on M_ValhallaFoliage (masked, two-sided). ~1.2k tris. Wind not done.</t>
         </is>
       </c>
     </row>
@@ -3002,12 +3027,12 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural rock</t>
+          <t>Opus 5.5 + Blender MCP: procedural rock</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
         <is>
-          <t>CC0 sandstone</t>
+          <t>CC0: Poly Haven old_sandstone_02 (SandstoneRock)</t>
         </is>
       </c>
       <c r="I44" s="1" t="inlineStr">
@@ -3022,7 +3047,12 @@
       </c>
       <c r="K44" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L44" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): Wind-carved sandstone boulder: bedding planes eroded into ledges, undercut foot, flattened top; strata run horizontal. First-pass bounds kept.</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3089,12 @@
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural modular</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>CC0 sandstone</t>
+          <t>CC0: Poly Haven sandstone_blocks_05 (SandstoneBlocks)</t>
         </is>
       </c>
       <c r="I45" s="1" t="inlineStr">
@@ -3079,12 +3109,12 @@
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L45" s="1" t="inlineStr">
         <is>
-          <t>Vision blockers</t>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): Dressed ashlar: projecting plinth, body, string course and individual capstones (a few worn lower); the end pier has a moulded cap and a low pyramid stone. Bounds identical to the first pass; VisionBlocker kept. Block joints do not line up across module seams (box UVs per module); not noticeable from the game camera.  (Earlier note: Vision blockers)</t>
         </is>
       </c>
     </row>
@@ -3865,12 +3895,12 @@
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: model + VFX</t>
+          <t>Opus 5.5 + Blender MCP: model</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>Procedural</t>
+          <t>MI_StoneWall plinth, MI_Rock obelisk, M_PortalGlow runes</t>
         </is>
       </c>
       <c r="I58" s="1" t="inlineStr">
@@ -3885,7 +3915,12 @@
       </c>
       <c r="K58" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L58" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave3_desert.py): Rune-stone: two-step octagonal plinth with a glowing ring inlay, tapering obelisk with a pyramidion and glowing rune bars on four faces. Same 1.21 m height, slightly smaller footprint; collision profile kept. M_PortalGlow toned down (EmissiveStrength 4 -&gt; 1.6, deeper violet) so it no longer blooms to white.</t>
         </is>
       </c>
     </row>
@@ -3984,12 +4019,12 @@
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>Rendered from the new 3D models in a Blender icon studio</t>
+          <t>Rendered from the game's own models in a Blender icon studio (wave4_icons.py)</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Materials rebuilt from the Unreal MIs (Import/UI/icon_materials.json)</t>
         </is>
       </c>
       <c r="I60" s="1" t="inlineStr">
@@ -4004,7 +4039,12 @@
       </c>
       <c r="K60" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L60" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5): 30 icons, 128 px with outline and shadow (wave4_icon_finish.py): every item in items.json. 22 re-rendered from the weapon/shield glb and MetaHuman armour FBX (same file names, so items.json and the web editor pick them up); 8 new (dagger_iron, totem_bone, ring_strength, ring_wisdom, potion_health, potion_mana, rat_tail, gold_coin, modelled in the studio) and set as inventoryIcon in items.json. The other 46 1.0 icons (32 px pixel art) belong to no current item and have no model; left as they are. Imported by import_ui_icons.py (bilinear + mips for 128 px, nearest for 32 px).</t>
         </is>
       </c>
     </row>
@@ -4041,12 +4081,12 @@
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>Blender-rendered emblems + painted frames</t>
+          <t>Procedural: signed-distance emblems shaded as raised metal (martial) or glowing light (spells) (wave4_skill_icons.py)</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Background washed in each skill's iconColor</t>
         </is>
       </c>
       <c r="I61" s="1" t="inlineStr">
@@ -4061,7 +4101,12 @@
       </c>
       <c r="K61" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L61" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5): 41 icons, one per skill in skills.json, in Import/UI/Icons/Skills/&lt;id&gt;.png -&gt; /Game/Valhalla/UI/Icons/Skills. The action bar and skills pane show them; a skill without one keeps the generated code tile.</t>
         </is>
       </c>
     </row>
@@ -4098,12 +4143,12 @@
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>Blender-rendered / procedural 2D</t>
+          <t>Procedural 2D (wave4_ui_frames.py)</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>CC0 materials</t>
+          <t>CC0 Leather (panel interior) + bronze / iron bevels</t>
         </is>
       </c>
       <c r="I62" s="1" t="inlineStr">
@@ -4118,12 +4163,12 @@
       </c>
       <c r="K62" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L62" s="1" t="inlineStr">
         <is>
-          <t>Pairs with B-07</t>
+          <t>Done 2026-09-24 (Opus 5.5): Nine-slice T_UI_Panel (leather in bronze trim, corner studs), T_UI_Slot (bronze rim, dark well), T_UI_Button, T_UI_BarFrame (iron), T_UI_BarFill (gloss ramp tinted by the bar colour) -&gt; /Game/Valhalla/UI/Frames. Applied to the current C++ HUD (MakePanel, MakeCell, MakeButton, MakeBar, combat log); B-07 can reuse them in a Widget Blueprint.  (Earlier note: Pairs with B-07)</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4329,7 @@
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
@@ -4304,12 +4349,12 @@
       </c>
       <c r="K65" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L65" s="1" t="inlineStr">
         <is>
-          <t>NWN staple</t>
+          <t>NWN staple. Done 2026-09-24 (Opus 5.5, wave5_kit.py Tavern): 64 cm wall, window and corner, 128 cm door, a 3.6 m two-storey build (stone ground floor, jettied timber-and-plaster upper floor), 128 x 128 slate gable roof, chimney, hanging sign, plank floor. In /Game/Valhalla/Environment/Tavern. Poly Haven SlateRoof, OakPlanks, DarkPlanks. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4391,7 @@
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
@@ -4366,7 +4411,12 @@
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L66" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py Temple): 2.4 m limestone wall and pilaster wall, fluted marble column, altar with candles and a gilt sun disc, steps, mosaic floor, brazier, a hooded statue. Braziers and altar candles burn with the animated M_ValhallaFire and get a flickering light from fire_lights.py. Poly Haven TempleStone, Marble, TempleFloor. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4453,7 @@
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
@@ -4423,7 +4473,12 @@
       </c>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L67" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py Keep): 50 cm curtain walls in 1.28 m modules (plain and arrow slit), corner pier, round tower (2.16 m across, 4.8 m tall), gatehouse with a raised portcullis, banner. The gate uses its own triangles for collision, so players walk through the open arch (capsule-tested); it has no closed state yet. Outside faces +Y. Poly Haven KeepStone. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4515,7 @@
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: modular + broken variants</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
@@ -4480,7 +4535,12 @@
       </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L68" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py Ruins): block-laid broken walls (ragged tops, every block supported), corner, low wall, snapped and fallen columns, half arch (walk-through), broken statue, rubble. Poly Haven RuinStone, MossyRock. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4577,7 @@
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
@@ -4537,7 +4597,12 @@
       </c>
       <c r="K69" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L69" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py River): humped stone bridge (3.84 m, 80 cm between the parapets), plank footbridge, river-bank edge strip and corner, reeds, stepping stones. Both bridges use their own triangles for collision and are walkable (capsule-tested). Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4639,7 @@
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural rock modular</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
@@ -4594,12 +4659,12 @@
       </c>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L70" s="1" t="inlineStr">
         <is>
-          <t>Needed for B-06</t>
+          <t>Needed for B-06. Done 2026-09-24 (Opus 5.5, wave5_kit.py Cave): ledged rock walls 1.28 x 0.64 x 2.4 m and 1.4 m, pillar to hide joints and turn corners, a ceiling lip that overhangs 0.9 m (no full roof, for the top-down camera), floor tile, stalagmites, stalactites, glowing crystals, rubble. Poly Haven CaveRock, CaveFloor. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4758,7 @@
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: models</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
@@ -4713,7 +4778,12 @@
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L72" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py Interior): bar counter, table, chair, bench, bed, shelf, books, candle, chest, keg, fireplace, table clutter. The fireplace and candle burn with the animated M_ValhallaFire and get a flickering light from fire_lights.py. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4750,7 +4820,7 @@
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: models</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
@@ -4770,12 +4840,12 @@
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L73" s="1" t="inlineStr">
         <is>
-          <t>EQ-style camps</t>
+          <t>EQ-style camps. Done 2026-09-24 (Opus 5.5, wave5_kit.py Camp): A-frame and bell tents, campfire, cooking fire (tripod and pot), bedroll, weapon rack, log seat, supply pile. Fires: animated M_ValhallaFire flames (rising noise, no shadow, no collision) plus a flickering PointLight per fire from fire_lights.add_all(). Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4882,7 @@
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: procedural foliage</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
@@ -4832,7 +4902,12 @@
       </c>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L74" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py Foliage): two bushes, grass tuft, two flower patches, fern, dead tree, stump, fallen log. Card materials (GrassTuft, Reeds, Fern, FlowersA/B, procedural, wave5_foliage_textures.py) on M_ValhallaFoliage; cards have no collision. No wind yet. Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>
@@ -4869,7 +4944,7 @@
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>Opus + Blender MCP: models</t>
+          <t>Opus 5.5 + Blender MCP: procedural (wave5_kit.py)</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
@@ -4889,7 +4964,12 @@
       </c>
       <c r="K75" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L75" s="0" t="inlineStr">
+        <is>
+          <t>Done 2026-09-24 (Opus 5.5, wave5_kit.py DesertVariety): half-buried ribcage and bones, horned skull, sandstone ruin wall and column, striped nomad awning with rug and cushions, pottery (amphorae, urn, shards). Review level /Game/Valhalla/Maps/Dev/L_ArtReview_Wave5.</t>
         </is>
       </c>
     </row>

</xml_diff>